<commit_message>
Add Punto de Equilibrio bullet chart with detail modal
New "Punto de Equilibrio por Departamento" card below Ventas por
Departamento / Concentración de Cartera. Per-department bullet bars show
Ingreso Neto (Monto PPTO aprobado, sin diferencial ni pausados) vs the
piso de venta target marker, colored by attainment (green/amber/red),
with a Mensual/Anual toggle (Anual = piso x12; Mensual = selected month
or monthly average). Break-even inputs are hardcoded from Escenario 2
(Social Media mapped to Digital). Clicking the chart opens a modal with
the full detail: assumptions block plus a per-department table (Costo
Fijo, Gasto Asignado, Gastos/mes, Piso mensual/anual, Ingreso Neto and
% cumplimiento) with totals.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Punto de equilibrio JUNIO.xlsx
+++ b/Punto de equilibrio JUNIO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario19\tablero-kacrea\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF333628-1FBC-4F93-9732-11B7F6B5E266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7518A4A4-CA55-42E6-ACB1-A75FFCF80445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{53FCD251-3E6B-4872-A7F8-153FC9D4EB64}"/>
   </bookViews>
@@ -96,7 +96,7 @@
     <t>Total</t>
   </si>
   <si>
-    <t>piso de venta Junio</t>
+    <t>piso de venta</t>
   </si>
 </sst>
 </file>
@@ -107,7 +107,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -152,6 +152,19 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -210,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -239,6 +252,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -643,7 +658,7 @@
       <c r="A8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="16">
         <v>2950</v>
       </c>
       <c r="C8" s="11">
@@ -675,7 +690,7 @@
       <c r="A9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="16">
         <v>2350</v>
       </c>
       <c r="C9" s="11">
@@ -707,7 +722,7 @@
       <c r="A10" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="16">
         <v>1800</v>
       </c>
       <c r="C10" s="11">
@@ -739,7 +754,7 @@
       <c r="A11" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="16">
         <v>1300</v>
       </c>
       <c r="C11" s="11">
@@ -771,7 +786,7 @@
       <c r="A12" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="16">
         <v>1800</v>
       </c>
       <c r="C12" s="11">
@@ -803,7 +818,7 @@
       <c r="A13" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="17">
         <v>10200</v>
       </c>
       <c r="C13" s="12">
@@ -837,5 +852,6 @@
     <mergeCell ref="G4:H4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Ingresos/Costo Variable/Mc Promedio columns to PE detail modal
The Punto de Equilibrio detail modal now shows the Escenario 2 columns
Ingresos Promedio, Costo Variable Promedio, Mc Promedio and % Margen de
Contribución per department (hardcoded from the scenario; Mc = Ingresos
- Costo Variable, % Mc = Mc/Ingresos), with matching totals. Values
match the Excel exactly.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Punto de equilibrio JUNIO.xlsx
+++ b/Punto de equilibrio JUNIO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario19\tablero-kacrea\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7518A4A4-CA55-42E6-ACB1-A75FFCF80445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A4A2F8-34AD-4B75-A4EC-1DF2D5DB7884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{53FCD251-3E6B-4872-A7F8-153FC9D4EB64}"/>
   </bookViews>
@@ -69,12 +69,6 @@
     <t>Costo Variable Promedio</t>
   </si>
   <si>
-    <t>Mc Promedio</t>
-  </si>
-  <si>
-    <t>%</t>
-  </si>
-  <si>
     <t>Punto de equilibrio</t>
   </si>
   <si>
@@ -97,6 +91,12 @@
   </si>
   <si>
     <t>piso de venta</t>
+  </si>
+  <si>
+    <t>Margen de contribución Promedio</t>
+  </si>
+  <si>
+    <t>% Margen de Contribución</t>
   </si>
 </sst>
 </file>
@@ -243,6 +243,8 @@
     <xf numFmtId="164" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -252,8 +254,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -578,18 +578,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -606,10 +606,10 @@
       <c r="C4" s="7">
         <v>13250</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="15"/>
+      <c r="H4" s="17"/>
       <c r="I4" s="8">
         <v>0.3</v>
       </c>
@@ -642,23 +642,23 @@
         <v>10</v>
       </c>
       <c r="G7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="J7" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="16">
+        <v>12</v>
+      </c>
+      <c r="B8" s="13">
         <v>2950</v>
       </c>
       <c r="C8" s="11">
@@ -677,7 +677,8 @@
         <v>3810.61</v>
       </c>
       <c r="H8" s="4">
-        <v>0.91</v>
+        <f>G8/E8</f>
+        <v>0.90945346062052512</v>
       </c>
       <c r="I8" s="9">
         <v>6157.54</v>
@@ -688,9 +689,9 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="16">
+        <v>13</v>
+      </c>
+      <c r="B9" s="13">
         <v>2350</v>
       </c>
       <c r="C9" s="11">
@@ -709,7 +710,8 @@
         <v>2454.96</v>
       </c>
       <c r="H9" s="4">
-        <v>0.96</v>
+        <f>G9/E9</f>
+        <v>0.95960598835163968</v>
       </c>
       <c r="I9" s="9">
         <v>5210.4799999999996</v>
@@ -720,9 +722,9 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="16">
+        <v>14</v>
+      </c>
+      <c r="B10" s="13">
         <v>1800</v>
       </c>
       <c r="C10" s="11">
@@ -741,7 +743,8 @@
         <v>4400.38</v>
       </c>
       <c r="H10" s="4">
-        <v>0.99</v>
+        <f t="shared" ref="H10:H12" si="0">G10/E10</f>
+        <v>0.99369734141169619</v>
       </c>
       <c r="I10" s="9">
         <v>4478.22</v>
@@ -752,9 +755,9 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="16">
+        <v>15</v>
+      </c>
+      <c r="B11" s="13">
         <v>1300</v>
       </c>
       <c r="C11" s="11">
@@ -773,7 +776,8 @@
         <v>2503.33</v>
       </c>
       <c r="H11" s="4">
-        <v>0.88</v>
+        <f t="shared" si="0"/>
+        <v>0.88015259123830958</v>
       </c>
       <c r="I11" s="9">
         <v>4487.8599999999997</v>
@@ -784,9 +788,9 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="16">
+        <v>16</v>
+      </c>
+      <c r="B12" s="13">
         <v>1800</v>
       </c>
       <c r="C12" s="11">
@@ -805,7 +809,8 @@
         <v>7368.59</v>
       </c>
       <c r="H12" s="4">
-        <v>0.31</v>
+        <f t="shared" si="0"/>
+        <v>0.31286831158475409</v>
       </c>
       <c r="I12" s="9">
         <v>14223.24</v>
@@ -816,9 +821,9 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="17">
+        <v>17</v>
+      </c>
+      <c r="B13" s="14">
         <v>10200</v>
       </c>
       <c r="C13" s="12">

</xml_diff>

<commit_message>
Update PE Escenario 2 figures from latest xlsx
Costos fijos, gastos, pisos de venta e ingresos/costo variable
promedio por departamento actualizados según el Excel de junio.
</commit_message>
<xml_diff>
--- a/Punto de equilibrio JUNIO.xlsx
+++ b/Punto de equilibrio JUNIO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario19\tablero-kacrea\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A4A2F8-34AD-4B75-A4EC-1DF2D5DB7884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45642047-1611-4B34-B443-90C6E3355263}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{53FCD251-3E6B-4872-A7F8-153FC9D4EB64}"/>
   </bookViews>
@@ -223,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -232,7 +232,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -578,39 +577,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="7">
-        <v>10200</v>
+      <c r="C3" s="6">
+        <v>9600</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="6">
         <v>13250</v>
       </c>
-      <c r="G4" s="17" t="s">
+      <c r="G4" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="17"/>
-      <c r="I4" s="8">
+      <c r="H4" s="16"/>
+      <c r="I4" s="7">
         <v>0.3</v>
       </c>
     </row>
@@ -618,8 +617,9 @@
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="7">
-        <v>23450</v>
+      <c r="C5" s="6">
+        <f>C3+C4</f>
+        <v>22850</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.3">
@@ -658,164 +658,164 @@
       <c r="A8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="13">
-        <v>2950</v>
-      </c>
-      <c r="C8" s="11">
+      <c r="B8" s="12">
+        <v>2700</v>
+      </c>
+      <c r="C8" s="10">
         <v>0.2</v>
       </c>
-      <c r="D8" s="9">
+      <c r="D8" s="8">
         <v>2650</v>
       </c>
-      <c r="E8" s="9">
-        <v>4190</v>
-      </c>
-      <c r="F8" s="9">
-        <v>379.39</v>
-      </c>
-      <c r="G8" s="9">
-        <v>3810.61</v>
+      <c r="E8" s="8">
+        <v>5025</v>
+      </c>
+      <c r="F8" s="8">
+        <v>442.07714799600643</v>
+      </c>
+      <c r="G8" s="8">
+        <v>4582.9228520039933</v>
       </c>
       <c r="H8" s="4">
         <f>G8/E8</f>
-        <v>0.90945346062052512</v>
-      </c>
-      <c r="I8" s="9">
-        <v>6157.54</v>
-      </c>
-      <c r="J8" s="9">
-        <v>6200</v>
+        <v>0.91202444815999861</v>
+      </c>
+      <c r="I8" s="8">
+        <v>5866.070817283</v>
+      </c>
+      <c r="J8" s="8">
+        <v>6000</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="13">
-        <v>2350</v>
-      </c>
-      <c r="C9" s="11">
+      <c r="B9" s="12">
+        <v>3400</v>
+      </c>
+      <c r="C9" s="10">
         <v>0.2</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="8">
         <v>2650</v>
       </c>
-      <c r="E9" s="9">
-        <v>2558.3000000000002</v>
-      </c>
-      <c r="F9" s="9">
-        <v>103.34</v>
-      </c>
-      <c r="G9" s="9">
-        <v>2454.96</v>
+      <c r="E9" s="8">
+        <v>3111.0835274402475</v>
+      </c>
+      <c r="F9" s="8">
+        <v>193.13666666666668</v>
+      </c>
+      <c r="G9" s="8">
+        <v>2917.9468607735807</v>
       </c>
       <c r="H9" s="4">
         <f>G9/E9</f>
-        <v>0.95960598835163968</v>
-      </c>
-      <c r="I9" s="9">
-        <v>5210.4799999999996</v>
-      </c>
-      <c r="J9" s="9">
-        <v>5300</v>
+        <v>0.93791980672869402</v>
+      </c>
+      <c r="I9" s="8">
+        <v>6450.444863832633</v>
+      </c>
+      <c r="J9" s="8">
+        <v>6500</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="13">
-        <v>1800</v>
-      </c>
-      <c r="C10" s="11">
+      <c r="B10" s="12">
+        <v>1400</v>
+      </c>
+      <c r="C10" s="10">
         <v>0.2</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="8">
         <v>2650</v>
       </c>
-      <c r="E10" s="9">
-        <v>4428.29</v>
-      </c>
-      <c r="F10" s="9">
-        <v>27.91</v>
-      </c>
-      <c r="G10" s="9">
-        <v>4400.38</v>
+      <c r="E10" s="8">
+        <v>4181.0758942218717</v>
+      </c>
+      <c r="F10" s="8">
+        <v>25.747230721393038</v>
+      </c>
+      <c r="G10" s="8">
+        <v>4155.3286635004788</v>
       </c>
       <c r="H10" s="4">
-        <f t="shared" ref="H10:H12" si="0">G10/E10</f>
-        <v>0.99369734141169619</v>
-      </c>
-      <c r="I10" s="9">
-        <v>4478.22</v>
-      </c>
-      <c r="J10" s="9">
-        <v>4500</v>
+        <f t="shared" ref="H10:H13" si="0">G10/E10</f>
+        <v>0.99384196044922912</v>
+      </c>
+      <c r="I10" s="8">
+        <v>4075.0945936810203</v>
+      </c>
+      <c r="J10" s="8">
+        <v>4100</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="13">
-        <v>1300</v>
-      </c>
-      <c r="C11" s="11">
+      <c r="B11" s="12">
+        <v>700</v>
+      </c>
+      <c r="C11" s="10">
         <v>0.2</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="8">
         <v>2650</v>
       </c>
-      <c r="E11" s="9">
-        <v>2844.2</v>
-      </c>
-      <c r="F11" s="9">
-        <v>340.87</v>
-      </c>
-      <c r="G11" s="9">
-        <v>2503.33</v>
+      <c r="E11" s="8">
+        <v>2628.5</v>
+      </c>
+      <c r="F11" s="8">
+        <v>405.30891337595108</v>
+      </c>
+      <c r="G11" s="8">
+        <v>2223.1910866240487</v>
       </c>
       <c r="H11" s="4">
         <f t="shared" si="0"/>
-        <v>0.88015259123830958</v>
-      </c>
-      <c r="I11" s="9">
-        <v>4487.8599999999997</v>
-      </c>
-      <c r="J11" s="9">
-        <v>4500</v>
+        <v>0.84580220149288521</v>
+      </c>
+      <c r="I11" s="8">
+        <v>3960.7369123502804</v>
+      </c>
+      <c r="J11" s="8">
+        <v>4000</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="13">
-        <v>1800</v>
-      </c>
-      <c r="C12" s="11">
+      <c r="B12" s="12">
+        <v>1400</v>
+      </c>
+      <c r="C12" s="10">
         <v>0.2</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="8">
         <v>2650</v>
       </c>
-      <c r="E12" s="9">
-        <v>23551.73</v>
-      </c>
-      <c r="F12" s="9">
-        <v>16183.14</v>
-      </c>
-      <c r="G12" s="9">
-        <v>7368.59</v>
+      <c r="E12" s="8">
+        <v>19915.974884756415</v>
+      </c>
+      <c r="F12" s="8">
+        <v>13780.641542038522</v>
+      </c>
+      <c r="G12" s="8">
+        <v>6135.3333427178932</v>
       </c>
       <c r="H12" s="4">
         <f t="shared" si="0"/>
-        <v>0.31286831158475409</v>
-      </c>
-      <c r="I12" s="9">
-        <v>14223.24</v>
-      </c>
-      <c r="J12" s="9">
+        <v>0.30806090980832906</v>
+      </c>
+      <c r="I12" s="8">
+        <v>13146.750759516519</v>
+      </c>
+      <c r="J12" s="8">
         <v>25000</v>
       </c>
     </row>
@@ -823,32 +823,39 @@
       <c r="A13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="14">
-        <v>10200</v>
-      </c>
-      <c r="C13" s="12">
+      <c r="B13" s="13">
+        <f>SUM(B8:B12)</f>
+        <v>9600</v>
+      </c>
+      <c r="C13" s="11">
         <v>1</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="9">
         <v>13250</v>
       </c>
-      <c r="E13" s="10">
-        <v>37572.51</v>
-      </c>
-      <c r="F13" s="10">
-        <v>17034.650000000001</v>
-      </c>
-      <c r="G13" s="10">
-        <v>20537.87</v>
-      </c>
-      <c r="H13" s="6">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="I13" s="10">
-        <v>34557.339999999997</v>
-      </c>
-      <c r="J13" s="10">
-        <v>45500</v>
+      <c r="E13" s="13">
+        <f>SUM(E8:E12)</f>
+        <v>34861.634306418535</v>
+      </c>
+      <c r="F13" s="13">
+        <f>SUM(F8:F12)</f>
+        <v>14846.911500798538</v>
+      </c>
+      <c r="G13" s="13">
+        <f>SUM(G8:G12)</f>
+        <v>20014.722805619997</v>
+      </c>
+      <c r="H13" s="4">
+        <f t="shared" si="0"/>
+        <v>0.57411889040253616</v>
+      </c>
+      <c r="I13" s="13">
+        <f>SUM(I8:I12)</f>
+        <v>33499.097946663453</v>
+      </c>
+      <c r="J13" s="13">
+        <f>SUM(J8:J12)</f>
+        <v>45600</v>
       </c>
     </row>
   </sheetData>
@@ -858,5 +865,8 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="H13" formula="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>